<commit_message>
fixed erros in write section
edit_existing was incomplete and was not working properly-- now fixed.. and improved output formatting of read in excel
</commit_message>
<xml_diff>
--- a/reading_data/names.xlsx
+++ b/reading_data/names.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" min="1" max="1"/>
@@ -532,6 +532,50 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nihal</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>nothin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>jamal</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>